<commit_message>
Pre-fill RM workbook with synthetic deals; add download link
- dump_deals.js: tiny Node script that loads pipeline/js/{config,data}.js
  in a vm context and dumps allDeals to deals.json
- build_workbook.py: now reads deals.json and pre-populates each RM tab
  with the dashboard's exact 76 deals (Customer, Product, Stage, Amount,
  Probability, Date Entered Stage, Expected Close as hard values; Days
  in Stage, Annual Rev, Weighted Rev remain formulas)
- Empty rows below each officer's deals still carry the formulas so RMs
  can add new entries and have them auto-populate
- pipeline/index.html: "RM Template" download link in the header pointing
  to templates/RM-pipeline-template.xlsx

https://claude.ai/code/session_01XW8PCjUB3Sv4m4W8pgSLGG
</commit_message>
<xml_diff>
--- a/pipeline/templates/RM-pipeline-template.xlsx
+++ b/pipeline/templates/RM-pipeline-template.xlsx
@@ -25,9 +25,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
-    <numFmt numFmtId="165" formatCode="m/d/yyyy"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="166" formatCode="m/d/yyyy"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -143,12 +144,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1344,17 +1345,37 @@
       </c>
     </row>
     <row r="3">
-      <c r="D3" s="6" t="n"/>
-      <c r="E3" s="12">
-        <f>IF(C3="","",VLOOKUP(C3,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F3" s="13" t="n"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Northstar Tech</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Deposits</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Qualified</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="n">
+        <v>1986780.75</v>
+      </c>
+      <c r="E3" s="12" t="n">
+        <v>0.2966</v>
+      </c>
+      <c r="F3" s="13" t="n">
+        <v>46158</v>
+      </c>
       <c r="G3" s="14">
         <f>IF(F3="","",TODAY()-F3)</f>
         <v/>
       </c>
-      <c r="H3" s="13" t="n"/>
+      <c r="H3" s="13" t="n">
+        <v>46331</v>
+      </c>
       <c r="I3" s="15">
         <f>IF(OR(B3="",D3=""),"",D3*VLOOKUP(B3,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -1365,20 +1386,37 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="16" t="n"/>
-      <c r="B4" s="16" t="n"/>
-      <c r="C4" s="16" t="n"/>
-      <c r="D4" s="17" t="n"/>
-      <c r="E4" s="12">
-        <f>IF(C4="","",VLOOKUP(C4,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F4" s="18" t="n"/>
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>Oakridge Auto</t>
+        </is>
+      </c>
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>Treasury Mgmt</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="D4" s="17" t="n">
+        <v>56255.38</v>
+      </c>
+      <c r="E4" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" s="18" t="n">
+        <v>46145</v>
+      </c>
       <c r="G4" s="14">
         <f>IF(F4="","",TODAY()-F4)</f>
         <v/>
       </c>
-      <c r="H4" s="18" t="n"/>
+      <c r="H4" s="18" t="n">
+        <v>46210</v>
+      </c>
       <c r="I4" s="15">
         <f>IF(OR(B4="",D4=""),"",D4*VLOOKUP(B4,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -1390,17 +1428,37 @@
       <c r="K4" s="16" t="n"/>
     </row>
     <row r="5">
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="12">
-        <f>IF(C5="","",VLOOKUP(C5,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F5" s="13" t="n"/>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Pacific Imports</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Treasury Mgmt</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Proposal</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>204686.79</v>
+      </c>
+      <c r="E5" s="12" t="n">
+        <v>0.5004</v>
+      </c>
+      <c r="F5" s="13" t="n">
+        <v>46138</v>
+      </c>
       <c r="G5" s="14">
         <f>IF(F5="","",TODAY()-F5)</f>
         <v/>
       </c>
-      <c r="H5" s="13" t="n"/>
+      <c r="H5" s="13" t="n">
+        <v>46280</v>
+      </c>
       <c r="I5" s="15">
         <f>IF(OR(B5="",D5=""),"",D5*VLOOKUP(B5,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -1411,20 +1469,37 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="n"/>
-      <c r="B6" s="16" t="n"/>
-      <c r="C6" s="16" t="n"/>
-      <c r="D6" s="17" t="n"/>
-      <c r="E6" s="12">
-        <f>IF(C6="","",VLOOKUP(C6,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F6" s="18" t="n"/>
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>Quartz Mining</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>Deposits</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="D6" s="17" t="n">
+        <v>779213.01</v>
+      </c>
+      <c r="E6" s="12" t="n">
+        <v>0.974</v>
+      </c>
+      <c r="F6" s="18" t="n">
+        <v>46187</v>
+      </c>
       <c r="G6" s="14">
         <f>IF(F6="","",TODAY()-F6)</f>
         <v/>
       </c>
-      <c r="H6" s="18" t="n"/>
+      <c r="H6" s="18" t="n">
+        <v>46231</v>
+      </c>
       <c r="I6" s="15">
         <f>IF(OR(B6="",D6=""),"",D6*VLOOKUP(B6,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -1436,17 +1511,37 @@
       <c r="K6" s="16" t="n"/>
     </row>
     <row r="7">
-      <c r="D7" s="6" t="n"/>
-      <c r="E7" s="12">
-        <f>IF(C7="","",VLOOKUP(C7,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F7" s="13" t="n"/>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Redwood Construction</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Deposits</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Qualified</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>2490783.84</v>
+      </c>
+      <c r="E7" s="12" t="n">
+        <v>0.2334</v>
+      </c>
+      <c r="F7" s="13" t="n">
+        <v>46128</v>
+      </c>
       <c r="G7" s="14">
         <f>IF(F7="","",TODAY()-F7)</f>
         <v/>
       </c>
-      <c r="H7" s="13" t="n"/>
+      <c r="H7" s="13" t="n">
+        <v>46351</v>
+      </c>
       <c r="I7" s="15">
         <f>IF(OR(B7="",D7=""),"",D7*VLOOKUP(B7,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -1457,20 +1552,37 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="n"/>
-      <c r="B8" s="16" t="n"/>
-      <c r="C8" s="16" t="n"/>
-      <c r="D8" s="17" t="n"/>
-      <c r="E8" s="12">
-        <f>IF(C8="","",VLOOKUP(C8,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F8" s="18" t="n"/>
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>Summit Hospitality</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>Other Fees</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>Qualified</t>
+        </is>
+      </c>
+      <c r="D8" s="17" t="n">
+        <v>56309.17</v>
+      </c>
+      <c r="E8" s="12" t="n">
+        <v>0.2152</v>
+      </c>
+      <c r="F8" s="18" t="n">
+        <v>46150</v>
+      </c>
       <c r="G8" s="14">
         <f>IF(F8="","",TODAY()-F8)</f>
         <v/>
       </c>
-      <c r="H8" s="18" t="n"/>
+      <c r="H8" s="18" t="n">
+        <v>46311</v>
+      </c>
       <c r="I8" s="15">
         <f>IF(OR(B8="",D8=""),"",D8*VLOOKUP(B8,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -1482,17 +1594,37 @@
       <c r="K8" s="16" t="n"/>
     </row>
     <row r="9">
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="12">
-        <f>IF(C9="","",VLOOKUP(C9,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F9" s="13" t="n"/>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Trinity Pharma</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Other Fees</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>36726.21</v>
+      </c>
+      <c r="E9" s="12" t="n">
+        <v>0.06569999999999999</v>
+      </c>
+      <c r="F9" s="13" t="n">
+        <v>46152</v>
+      </c>
       <c r="G9" s="14">
         <f>IF(F9="","",TODAY()-F9)</f>
         <v/>
       </c>
-      <c r="H9" s="13" t="n"/>
+      <c r="H9" s="13" t="n">
+        <v>46330</v>
+      </c>
       <c r="I9" s="15">
         <f>IF(OR(B9="",D9=""),"",D9*VLOOKUP(B9,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -1503,20 +1635,37 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="n"/>
-      <c r="B10" s="16" t="n"/>
-      <c r="C10" s="16" t="n"/>
-      <c r="D10" s="17" t="n"/>
-      <c r="E10" s="12">
-        <f>IF(C10="","",VLOOKUP(C10,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F10" s="18" t="n"/>
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t>Union Distributors</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>Comm Loan</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="inlineStr">
+        <is>
+          <t>Qualified</t>
+        </is>
+      </c>
+      <c r="D10" s="17" t="n">
+        <v>1681430.41</v>
+      </c>
+      <c r="E10" s="12" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="F10" s="18" t="n">
+        <v>46115</v>
+      </c>
       <c r="G10" s="14">
         <f>IF(F10="","",TODAY()-F10)</f>
         <v/>
       </c>
-      <c r="H10" s="18" t="n"/>
+      <c r="H10" s="18" t="n">
+        <v>46332</v>
+      </c>
       <c r="I10" s="15">
         <f>IF(OR(B10="",D10=""),"",D10*VLOOKUP(B10,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -1528,17 +1677,37 @@
       <c r="K10" s="16" t="n"/>
     </row>
     <row r="11">
-      <c r="D11" s="6" t="n"/>
-      <c r="E11" s="12">
-        <f>IF(C11="","",VLOOKUP(C11,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F11" s="13" t="n"/>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Vanguard Plastics</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Deposits</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>1591906.93</v>
+      </c>
+      <c r="E11" s="12" t="n">
+        <v>0.7977</v>
+      </c>
+      <c r="F11" s="13" t="n">
+        <v>46156</v>
+      </c>
       <c r="G11" s="14">
         <f>IF(F11="","",TODAY()-F11)</f>
         <v/>
       </c>
-      <c r="H11" s="13" t="n"/>
+      <c r="H11" s="13" t="n">
+        <v>46263</v>
+      </c>
       <c r="I11" s="15">
         <f>IF(OR(B11="",D11=""),"",D11*VLOOKUP(B11,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -1549,20 +1718,37 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="16" t="n"/>
-      <c r="B12" s="16" t="n"/>
-      <c r="C12" s="16" t="n"/>
-      <c r="D12" s="17" t="n"/>
-      <c r="E12" s="12">
-        <f>IF(C12="","",VLOOKUP(C12,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F12" s="18" t="n"/>
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>Westfield Retail</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>Deposits</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="D12" s="17" t="n">
+        <v>5644082.34</v>
+      </c>
+      <c r="E12" s="12" t="n">
+        <v>0.0905</v>
+      </c>
+      <c r="F12" s="18" t="n">
+        <v>46165</v>
+      </c>
       <c r="G12" s="14">
         <f>IF(F12="","",TODAY()-F12)</f>
         <v/>
       </c>
-      <c r="H12" s="18" t="n"/>
+      <c r="H12" s="18" t="n">
+        <v>46380</v>
+      </c>
       <c r="I12" s="15">
         <f>IF(OR(B12="",D12=""),"",D12*VLOOKUP(B12,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -1574,17 +1760,37 @@
       <c r="K12" s="16" t="n"/>
     </row>
     <row r="13">
-      <c r="D13" s="6" t="n"/>
-      <c r="E13" s="12">
-        <f>IF(C13="","",VLOOKUP(C13,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F13" s="13" t="n"/>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Yellowstone Ranch</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Comm Loan</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>2214860.59</v>
+      </c>
+      <c r="E13" s="12" t="n">
+        <v>0.1229</v>
+      </c>
+      <c r="F13" s="13" t="n">
+        <v>46158</v>
+      </c>
       <c r="G13" s="14">
         <f>IF(F13="","",TODAY()-F13)</f>
         <v/>
       </c>
-      <c r="H13" s="13" t="n"/>
+      <c r="H13" s="13" t="n">
+        <v>46358</v>
+      </c>
       <c r="I13" s="15">
         <f>IF(OR(B13="",D13=""),"",D13*VLOOKUP(B13,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -1595,20 +1801,37 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="16" t="n"/>
-      <c r="B14" s="16" t="n"/>
-      <c r="C14" s="16" t="n"/>
-      <c r="D14" s="17" t="n"/>
-      <c r="E14" s="12">
-        <f>IF(C14="","",VLOOKUP(C14,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F14" s="18" t="n"/>
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>Zenith Software</t>
+        </is>
+      </c>
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>Deposits</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="D14" s="17" t="n">
+        <v>631615.27</v>
+      </c>
+      <c r="E14" s="12" t="n">
+        <v>0.1412</v>
+      </c>
+      <c r="F14" s="18" t="n">
+        <v>46179</v>
+      </c>
       <c r="G14" s="14">
         <f>IF(F14="","",TODAY()-F14)</f>
         <v/>
       </c>
-      <c r="H14" s="18" t="n"/>
+      <c r="H14" s="18" t="n">
+        <v>46364</v>
+      </c>
       <c r="I14" s="15">
         <f>IF(OR(B14="",D14=""),"",D14*VLOOKUP(B14,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -1620,17 +1843,37 @@
       <c r="K14" s="16" t="n"/>
     </row>
     <row r="15">
-      <c r="D15" s="6" t="n"/>
-      <c r="E15" s="12">
-        <f>IF(C15="","",VLOOKUP(C15,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F15" s="13" t="n"/>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Alamo Equipment</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Comm Loan</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>815121.37</v>
+      </c>
+      <c r="E15" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" s="13" t="n">
+        <v>46166</v>
+      </c>
       <c r="G15" s="14">
         <f>IF(F15="","",TODAY()-F15)</f>
         <v/>
       </c>
-      <c r="H15" s="13" t="n"/>
+      <c r="H15" s="13" t="n">
+        <v>46242</v>
+      </c>
       <c r="I15" s="15">
         <f>IF(OR(B15="",D15=""),"",D15*VLOOKUP(B15,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -1641,20 +1884,37 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="16" t="n"/>
-      <c r="B16" s="16" t="n"/>
-      <c r="C16" s="16" t="n"/>
-      <c r="D16" s="17" t="n"/>
-      <c r="E16" s="12">
-        <f>IF(C16="","",VLOOKUP(C16,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F16" s="18" t="n"/>
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>Brazos Petroleum</t>
+        </is>
+      </c>
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>Treasury Mgmt</t>
+        </is>
+      </c>
+      <c r="C16" s="16" t="inlineStr">
+        <is>
+          <t>Proposal</t>
+        </is>
+      </c>
+      <c r="D16" s="17" t="n">
+        <v>258735.19</v>
+      </c>
+      <c r="E16" s="12" t="n">
+        <v>0.4877</v>
+      </c>
+      <c r="F16" s="18" t="n">
+        <v>46186</v>
+      </c>
       <c r="G16" s="14">
         <f>IF(F16="","",TODAY()-F16)</f>
         <v/>
       </c>
-      <c r="H16" s="18" t="n"/>
+      <c r="H16" s="18" t="n">
+        <v>46264</v>
+      </c>
       <c r="I16" s="15">
         <f>IF(OR(B16="",D16=""),"",D16*VLOOKUP(B16,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -2154,17 +2414,37 @@
       </c>
     </row>
     <row r="3">
-      <c r="D3" s="6" t="n"/>
-      <c r="E3" s="12">
-        <f>IF(C3="","",VLOOKUP(C3,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F3" s="13" t="n"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Zenith Software</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Deposits</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="n">
+        <v>3805889.47</v>
+      </c>
+      <c r="E3" s="12" t="n">
+        <v>0.1462</v>
+      </c>
+      <c r="F3" s="13" t="n">
+        <v>46115</v>
+      </c>
       <c r="G3" s="14">
         <f>IF(F3="","",TODAY()-F3)</f>
         <v/>
       </c>
-      <c r="H3" s="13" t="n"/>
+      <c r="H3" s="13" t="n">
+        <v>46383</v>
+      </c>
       <c r="I3" s="15">
         <f>IF(OR(B3="",D3=""),"",D3*VLOOKUP(B3,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -2175,20 +2455,37 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="16" t="n"/>
-      <c r="B4" s="16" t="n"/>
-      <c r="C4" s="16" t="n"/>
-      <c r="D4" s="17" t="n"/>
-      <c r="E4" s="12">
-        <f>IF(C4="","",VLOOKUP(C4,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F4" s="18" t="n"/>
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>Alamo Equipment</t>
+        </is>
+      </c>
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>Other Fees</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="D4" s="17" t="n">
+        <v>44796.73</v>
+      </c>
+      <c r="E4" s="12" t="n">
+        <v>0.0978</v>
+      </c>
+      <c r="F4" s="18" t="n">
+        <v>46113</v>
+      </c>
       <c r="G4" s="14">
         <f>IF(F4="","",TODAY()-F4)</f>
         <v/>
       </c>
-      <c r="H4" s="18" t="n"/>
+      <c r="H4" s="18" t="n">
+        <v>46336</v>
+      </c>
       <c r="I4" s="15">
         <f>IF(OR(B4="",D4=""),"",D4*VLOOKUP(B4,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -2200,17 +2497,37 @@
       <c r="K4" s="16" t="n"/>
     </row>
     <row r="5">
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="12">
-        <f>IF(C5="","",VLOOKUP(C5,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F5" s="13" t="n"/>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Brazos Petroleum</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Other Fees</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>21234.43</v>
+      </c>
+      <c r="E5" s="12" t="n">
+        <v>0.7959000000000001</v>
+      </c>
+      <c r="F5" s="13" t="n">
+        <v>46188</v>
+      </c>
       <c r="G5" s="14">
         <f>IF(F5="","",TODAY()-F5)</f>
         <v/>
       </c>
-      <c r="H5" s="13" t="n"/>
+      <c r="H5" s="13" t="n">
+        <v>46244</v>
+      </c>
       <c r="I5" s="15">
         <f>IF(OR(B5="",D5=""),"",D5*VLOOKUP(B5,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -2221,20 +2538,37 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="n"/>
-      <c r="B6" s="16" t="n"/>
-      <c r="C6" s="16" t="n"/>
-      <c r="D6" s="17" t="n"/>
-      <c r="E6" s="12">
-        <f>IF(C6="","",VLOOKUP(C6,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F6" s="18" t="n"/>
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>Cedar Cabinetry</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>Deposits</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>Qualified</t>
+        </is>
+      </c>
+      <c r="D6" s="17" t="n">
+        <v>664568.04</v>
+      </c>
+      <c r="E6" s="12" t="n">
+        <v>0.2805</v>
+      </c>
+      <c r="F6" s="18" t="n">
+        <v>46184</v>
+      </c>
       <c r="G6" s="14">
         <f>IF(F6="","",TODAY()-F6)</f>
         <v/>
       </c>
-      <c r="H6" s="18" t="n"/>
+      <c r="H6" s="18" t="n">
+        <v>46339</v>
+      </c>
       <c r="I6" s="15">
         <f>IF(OR(B6="",D6=""),"",D6*VLOOKUP(B6,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -2246,17 +2580,37 @@
       <c r="K6" s="16" t="n"/>
     </row>
     <row r="7">
-      <c r="D7" s="6" t="n"/>
-      <c r="E7" s="12">
-        <f>IF(C7="","",VLOOKUP(C7,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F7" s="13" t="n"/>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Driftwood Hotels</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Other Fees</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Proposal</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>51592.1</v>
+      </c>
+      <c r="E7" s="12" t="n">
+        <v>0.5394</v>
+      </c>
+      <c r="F7" s="13" t="n">
+        <v>46175</v>
+      </c>
       <c r="G7" s="14">
         <f>IF(F7="","",TODAY()-F7)</f>
         <v/>
       </c>
-      <c r="H7" s="13" t="n"/>
+      <c r="H7" s="13" t="n">
+        <v>46310</v>
+      </c>
       <c r="I7" s="15">
         <f>IF(OR(B7="",D7=""),"",D7*VLOOKUP(B7,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -2267,20 +2621,37 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="n"/>
-      <c r="B8" s="16" t="n"/>
-      <c r="C8" s="16" t="n"/>
-      <c r="D8" s="17" t="n"/>
-      <c r="E8" s="12">
-        <f>IF(C8="","",VLOOKUP(C8,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F8" s="18" t="n"/>
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>Acme Holdings</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>Deposits</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="D8" s="17" t="n">
+        <v>5523470.11</v>
+      </c>
+      <c r="E8" s="12" t="n">
+        <v>0.7583</v>
+      </c>
+      <c r="F8" s="18" t="n">
+        <v>46130</v>
+      </c>
       <c r="G8" s="14">
         <f>IF(F8="","",TODAY()-F8)</f>
         <v/>
       </c>
-      <c r="H8" s="18" t="n"/>
+      <c r="H8" s="18" t="n">
+        <v>46253</v>
+      </c>
       <c r="I8" s="15">
         <f>IF(OR(B8="",D8=""),"",D8*VLOOKUP(B8,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -2292,17 +2663,37 @@
       <c r="K8" s="16" t="n"/>
     </row>
     <row r="9">
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="12">
-        <f>IF(C9="","",VLOOKUP(C9,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F9" s="13" t="n"/>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Beacon Industries</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Treasury Mgmt</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Proposal</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>154984.05</v>
+      </c>
+      <c r="E9" s="12" t="n">
+        <v>0.5372</v>
+      </c>
+      <c r="F9" s="13" t="n">
+        <v>46123</v>
+      </c>
       <c r="G9" s="14">
         <f>IF(F9="","",TODAY()-F9)</f>
         <v/>
       </c>
-      <c r="H9" s="13" t="n"/>
+      <c r="H9" s="13" t="n">
+        <v>46286</v>
+      </c>
       <c r="I9" s="15">
         <f>IF(OR(B9="",D9=""),"",D9*VLOOKUP(B9,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -2313,20 +2704,37 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="n"/>
-      <c r="B10" s="16" t="n"/>
-      <c r="C10" s="16" t="n"/>
-      <c r="D10" s="17" t="n"/>
-      <c r="E10" s="12">
-        <f>IF(C10="","",VLOOKUP(C10,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F10" s="18" t="n"/>
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t>Cypress Group</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>Comm Loan</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="D10" s="17" t="n">
+        <v>1294674.45</v>
+      </c>
+      <c r="E10" s="12" t="n">
+        <v>0.1322</v>
+      </c>
+      <c r="F10" s="18" t="n">
+        <v>46140</v>
+      </c>
       <c r="G10" s="14">
         <f>IF(F10="","",TODAY()-F10)</f>
         <v/>
       </c>
-      <c r="H10" s="18" t="n"/>
+      <c r="H10" s="18" t="n">
+        <v>46364</v>
+      </c>
       <c r="I10" s="15">
         <f>IF(OR(B10="",D10=""),"",D10*VLOOKUP(B10,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -2338,17 +2746,37 @@
       <c r="K10" s="16" t="n"/>
     </row>
     <row r="11">
-      <c r="D11" s="6" t="n"/>
-      <c r="E11" s="12">
-        <f>IF(C11="","",VLOOKUP(C11,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F11" s="13" t="n"/>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Delta Manufacturing</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Comm Loan</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>670519.5699999999</v>
+      </c>
+      <c r="E11" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="13" t="n">
+        <v>46192</v>
+      </c>
       <c r="G11" s="14">
         <f>IF(F11="","",TODAY()-F11)</f>
         <v/>
       </c>
-      <c r="H11" s="13" t="n"/>
+      <c r="H11" s="13" t="n">
+        <v>46216</v>
+      </c>
       <c r="I11" s="15">
         <f>IF(OR(B11="",D11=""),"",D11*VLOOKUP(B11,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -2359,20 +2787,37 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="16" t="n"/>
-      <c r="B12" s="16" t="n"/>
-      <c r="C12" s="16" t="n"/>
-      <c r="D12" s="17" t="n"/>
-      <c r="E12" s="12">
-        <f>IF(C12="","",VLOOKUP(C12,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F12" s="18" t="n"/>
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>Evergreen Realty</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>Comm Loan</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="D12" s="17" t="n">
+        <v>7093495.94</v>
+      </c>
+      <c r="E12" s="12" t="n">
+        <v>0.8165</v>
+      </c>
+      <c r="F12" s="18" t="n">
+        <v>46150</v>
+      </c>
       <c r="G12" s="14">
         <f>IF(F12="","",TODAY()-F12)</f>
         <v/>
       </c>
-      <c r="H12" s="18" t="n"/>
+      <c r="H12" s="18" t="n">
+        <v>46262</v>
+      </c>
       <c r="I12" s="15">
         <f>IF(OR(B12="",D12=""),"",D12*VLOOKUP(B12,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -2384,17 +2829,37 @@
       <c r="K12" s="16" t="n"/>
     </row>
     <row r="13">
-      <c r="D13" s="6" t="n"/>
-      <c r="E13" s="12">
-        <f>IF(C13="","",VLOOKUP(C13,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F13" s="13" t="n"/>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Galleon Logistics</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Comm Loan</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Qualified</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>3025189.44</v>
+      </c>
+      <c r="E13" s="12" t="n">
+        <v>0.259</v>
+      </c>
+      <c r="F13" s="13" t="n">
+        <v>46174</v>
+      </c>
       <c r="G13" s="14">
         <f>IF(F13="","",TODAY()-F13)</f>
         <v/>
       </c>
-      <c r="H13" s="13" t="n"/>
+      <c r="H13" s="13" t="n">
+        <v>46328</v>
+      </c>
       <c r="I13" s="15">
         <f>IF(OR(B13="",D13=""),"",D13*VLOOKUP(B13,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -2405,20 +2870,37 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="16" t="n"/>
-      <c r="B14" s="16" t="n"/>
-      <c r="C14" s="16" t="n"/>
-      <c r="D14" s="17" t="n"/>
-      <c r="E14" s="12">
-        <f>IF(C14="","",VLOOKUP(C14,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F14" s="18" t="n"/>
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>Harbor Partners</t>
+        </is>
+      </c>
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>Treasury Mgmt</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="inlineStr">
+        <is>
+          <t>Qualified</t>
+        </is>
+      </c>
+      <c r="D14" s="17" t="n">
+        <v>118290.88</v>
+      </c>
+      <c r="E14" s="12" t="n">
+        <v>0.2855</v>
+      </c>
+      <c r="F14" s="18" t="n">
+        <v>46170</v>
+      </c>
       <c r="G14" s="14">
         <f>IF(F14="","",TODAY()-F14)</f>
         <v/>
       </c>
-      <c r="H14" s="18" t="n"/>
+      <c r="H14" s="18" t="n">
+        <v>46295</v>
+      </c>
       <c r="I14" s="15">
         <f>IF(OR(B14="",D14=""),"",D14*VLOOKUP(B14,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -2430,17 +2912,37 @@
       <c r="K14" s="16" t="n"/>
     </row>
     <row r="15">
-      <c r="D15" s="6" t="n"/>
-      <c r="E15" s="12">
-        <f>IF(C15="","",VLOOKUP(C15,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F15" s="13" t="n"/>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Ironwood Capital</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Comm Loan</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>652838.6800000001</v>
+      </c>
+      <c r="E15" s="12" t="n">
+        <v>0.0863</v>
+      </c>
+      <c r="F15" s="13" t="n">
+        <v>46175</v>
+      </c>
       <c r="G15" s="14">
         <f>IF(F15="","",TODAY()-F15)</f>
         <v/>
       </c>
-      <c r="H15" s="13" t="n"/>
+      <c r="H15" s="13" t="n">
+        <v>46368</v>
+      </c>
       <c r="I15" s="15">
         <f>IF(OR(B15="",D15=""),"",D15*VLOOKUP(B15,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -2451,20 +2953,37 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="16" t="n"/>
-      <c r="B16" s="16" t="n"/>
-      <c r="C16" s="16" t="n"/>
-      <c r="D16" s="17" t="n"/>
-      <c r="E16" s="12">
-        <f>IF(C16="","",VLOOKUP(C16,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F16" s="18" t="n"/>
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>Juniper Foods</t>
+        </is>
+      </c>
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>Comm Loan</t>
+        </is>
+      </c>
+      <c r="C16" s="16" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="D16" s="17" t="n">
+        <v>1212020.72</v>
+      </c>
+      <c r="E16" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="18" t="n">
+        <v>46169</v>
+      </c>
       <c r="G16" s="14">
         <f>IF(F16="","",TODAY()-F16)</f>
         <v/>
       </c>
-      <c r="H16" s="18" t="n"/>
+      <c r="H16" s="18" t="n">
+        <v>46229</v>
+      </c>
       <c r="I16" s="15">
         <f>IF(OR(B16="",D16=""),"",D16*VLOOKUP(B16,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -2964,17 +3483,37 @@
       </c>
     </row>
     <row r="3">
-      <c r="D3" s="6" t="n"/>
-      <c r="E3" s="12">
-        <f>IF(C3="","",VLOOKUP(C3,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F3" s="13" t="n"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Cedar Cabinetry</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Comm Loan</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="n">
+        <v>1005286.41</v>
+      </c>
+      <c r="E3" s="12" t="n">
+        <v>0.0581</v>
+      </c>
+      <c r="F3" s="13" t="n">
+        <v>46129</v>
+      </c>
       <c r="G3" s="14">
         <f>IF(F3="","",TODAY()-F3)</f>
         <v/>
       </c>
-      <c r="H3" s="13" t="n"/>
+      <c r="H3" s="13" t="n">
+        <v>46337</v>
+      </c>
       <c r="I3" s="15">
         <f>IF(OR(B3="",D3=""),"",D3*VLOOKUP(B3,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -2985,20 +3524,37 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="16" t="n"/>
-      <c r="B4" s="16" t="n"/>
-      <c r="C4" s="16" t="n"/>
-      <c r="D4" s="17" t="n"/>
-      <c r="E4" s="12">
-        <f>IF(C4="","",VLOOKUP(C4,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F4" s="18" t="n"/>
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>Driftwood Hotels</t>
+        </is>
+      </c>
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>Treasury Mgmt</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="D4" s="17" t="n">
+        <v>76930.69</v>
+      </c>
+      <c r="E4" s="12" t="n">
+        <v>0.764</v>
+      </c>
+      <c r="F4" s="18" t="n">
+        <v>46120</v>
+      </c>
       <c r="G4" s="14">
         <f>IF(F4="","",TODAY()-F4)</f>
         <v/>
       </c>
-      <c r="H4" s="18" t="n"/>
+      <c r="H4" s="18" t="n">
+        <v>46269</v>
+      </c>
       <c r="I4" s="15">
         <f>IF(OR(B4="",D4=""),"",D4*VLOOKUP(B4,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -3010,17 +3566,37 @@
       <c r="K4" s="16" t="n"/>
     </row>
     <row r="5">
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="12">
-        <f>IF(C5="","",VLOOKUP(C5,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F5" s="13" t="n"/>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Acme Holdings</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Comm Loan</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Qualified</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>8942929.720000001</v>
+      </c>
+      <c r="E5" s="12" t="n">
+        <v>0.2501</v>
+      </c>
+      <c r="F5" s="13" t="n">
+        <v>46163</v>
+      </c>
       <c r="G5" s="14">
         <f>IF(F5="","",TODAY()-F5)</f>
         <v/>
       </c>
-      <c r="H5" s="13" t="n"/>
+      <c r="H5" s="13" t="n">
+        <v>46326</v>
+      </c>
       <c r="I5" s="15">
         <f>IF(OR(B5="",D5=""),"",D5*VLOOKUP(B5,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -3031,20 +3607,37 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="n"/>
-      <c r="B6" s="16" t="n"/>
-      <c r="C6" s="16" t="n"/>
-      <c r="D6" s="17" t="n"/>
-      <c r="E6" s="12">
-        <f>IF(C6="","",VLOOKUP(C6,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F6" s="18" t="n"/>
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>Beacon Industries</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>Deposits</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="D6" s="17" t="n">
+        <v>2437446.78</v>
+      </c>
+      <c r="E6" s="12" t="n">
+        <v>0.1449</v>
+      </c>
+      <c r="F6" s="18" t="n">
+        <v>46192</v>
+      </c>
       <c r="G6" s="14">
         <f>IF(F6="","",TODAY()-F6)</f>
         <v/>
       </c>
-      <c r="H6" s="18" t="n"/>
+      <c r="H6" s="18" t="n">
+        <v>46330</v>
+      </c>
       <c r="I6" s="15">
         <f>IF(OR(B6="",D6=""),"",D6*VLOOKUP(B6,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -3056,17 +3649,37 @@
       <c r="K6" s="16" t="n"/>
     </row>
     <row r="7">
-      <c r="D7" s="6" t="n"/>
-      <c r="E7" s="12">
-        <f>IF(C7="","",VLOOKUP(C7,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F7" s="13" t="n"/>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Cypress Group</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Comm Loan</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Proposal</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>6584533.2</v>
+      </c>
+      <c r="E7" s="12" t="n">
+        <v>0.4954</v>
+      </c>
+      <c r="F7" s="13" t="n">
+        <v>46134</v>
+      </c>
       <c r="G7" s="14">
         <f>IF(F7="","",TODAY()-F7)</f>
         <v/>
       </c>
-      <c r="H7" s="13" t="n"/>
+      <c r="H7" s="13" t="n">
+        <v>46298</v>
+      </c>
       <c r="I7" s="15">
         <f>IF(OR(B7="",D7=""),"",D7*VLOOKUP(B7,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -3077,20 +3690,37 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="n"/>
-      <c r="B8" s="16" t="n"/>
-      <c r="C8" s="16" t="n"/>
-      <c r="D8" s="17" t="n"/>
-      <c r="E8" s="12">
-        <f>IF(C8="","",VLOOKUP(C8,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F8" s="18" t="n"/>
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>Delta Manufacturing</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>Other Fees</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>Qualified</t>
+        </is>
+      </c>
+      <c r="D8" s="17" t="n">
+        <v>26664.61</v>
+      </c>
+      <c r="E8" s="12" t="n">
+        <v>0.2668</v>
+      </c>
+      <c r="F8" s="18" t="n">
+        <v>46183</v>
+      </c>
       <c r="G8" s="14">
         <f>IF(F8="","",TODAY()-F8)</f>
         <v/>
       </c>
-      <c r="H8" s="18" t="n"/>
+      <c r="H8" s="18" t="n">
+        <v>46350</v>
+      </c>
       <c r="I8" s="15">
         <f>IF(OR(B8="",D8=""),"",D8*VLOOKUP(B8,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -3102,17 +3732,37 @@
       <c r="K8" s="16" t="n"/>
     </row>
     <row r="9">
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="12">
-        <f>IF(C9="","",VLOOKUP(C9,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F9" s="13" t="n"/>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Evergreen Realty</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Other Fees</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Proposal</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>67794</v>
+      </c>
+      <c r="E9" s="12" t="n">
+        <v>0.5078</v>
+      </c>
+      <c r="F9" s="13" t="n">
+        <v>46193</v>
+      </c>
       <c r="G9" s="14">
         <f>IF(F9="","",TODAY()-F9)</f>
         <v/>
       </c>
-      <c r="H9" s="13" t="n"/>
+      <c r="H9" s="13" t="n">
+        <v>46274</v>
+      </c>
       <c r="I9" s="15">
         <f>IF(OR(B9="",D9=""),"",D9*VLOOKUP(B9,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -3123,20 +3773,37 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="n"/>
-      <c r="B10" s="16" t="n"/>
-      <c r="C10" s="16" t="n"/>
-      <c r="D10" s="17" t="n"/>
-      <c r="E10" s="12">
-        <f>IF(C10="","",VLOOKUP(C10,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F10" s="18" t="n"/>
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t>Fairfield Energy</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>Deposits</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="D10" s="17" t="n">
+        <v>713863.45</v>
+      </c>
+      <c r="E10" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="18" t="n">
+        <v>46164</v>
+      </c>
       <c r="G10" s="14">
         <f>IF(F10="","",TODAY()-F10)</f>
         <v/>
       </c>
-      <c r="H10" s="18" t="n"/>
+      <c r="H10" s="18" t="n">
+        <v>46228</v>
+      </c>
       <c r="I10" s="15">
         <f>IF(OR(B10="",D10=""),"",D10*VLOOKUP(B10,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -3148,17 +3815,37 @@
       <c r="K10" s="16" t="n"/>
     </row>
     <row r="11">
-      <c r="D11" s="6" t="n"/>
-      <c r="E11" s="12">
-        <f>IF(C11="","",VLOOKUP(C11,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F11" s="13" t="n"/>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Galleon Logistics</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Comm Loan</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Proposal</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>4952275.33</v>
+      </c>
+      <c r="E11" s="12" t="n">
+        <v>0.5301</v>
+      </c>
+      <c r="F11" s="13" t="n">
+        <v>46191</v>
+      </c>
       <c r="G11" s="14">
         <f>IF(F11="","",TODAY()-F11)</f>
         <v/>
       </c>
-      <c r="H11" s="13" t="n"/>
+      <c r="H11" s="13" t="n">
+        <v>46313</v>
+      </c>
       <c r="I11" s="15">
         <f>IF(OR(B11="",D11=""),"",D11*VLOOKUP(B11,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -3169,20 +3856,37 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="16" t="n"/>
-      <c r="B12" s="16" t="n"/>
-      <c r="C12" s="16" t="n"/>
-      <c r="D12" s="17" t="n"/>
-      <c r="E12" s="12">
-        <f>IF(C12="","",VLOOKUP(C12,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F12" s="18" t="n"/>
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>Harbor Partners</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>Comm Loan</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="D12" s="17" t="n">
+        <v>16637851.99</v>
+      </c>
+      <c r="E12" s="12" t="n">
+        <v>0.1183</v>
+      </c>
+      <c r="F12" s="18" t="n">
+        <v>46145</v>
+      </c>
       <c r="G12" s="14">
         <f>IF(F12="","",TODAY()-F12)</f>
         <v/>
       </c>
-      <c r="H12" s="18" t="n"/>
+      <c r="H12" s="18" t="n">
+        <v>46370</v>
+      </c>
       <c r="I12" s="15">
         <f>IF(OR(B12="",D12=""),"",D12*VLOOKUP(B12,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -3194,17 +3898,37 @@
       <c r="K12" s="16" t="n"/>
     </row>
     <row r="13">
-      <c r="D13" s="6" t="n"/>
-      <c r="E13" s="12">
-        <f>IF(C13="","",VLOOKUP(C13,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F13" s="13" t="n"/>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Harbor Partners</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Deposits</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>2865543.02</v>
+      </c>
+      <c r="E13" s="12" t="n">
+        <v>0.1356</v>
+      </c>
+      <c r="F13" s="13" t="n">
+        <v>46138</v>
+      </c>
       <c r="G13" s="14">
         <f>IF(F13="","",TODAY()-F13)</f>
         <v/>
       </c>
-      <c r="H13" s="13" t="n"/>
+      <c r="H13" s="13" t="n">
+        <v>46326</v>
+      </c>
       <c r="I13" s="15">
         <f>IF(OR(B13="",D13=""),"",D13*VLOOKUP(B13,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -3774,17 +4498,37 @@
       </c>
     </row>
     <row r="3">
-      <c r="D3" s="6" t="n"/>
-      <c r="E3" s="12">
-        <f>IF(C3="","",VLOOKUP(C3,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F3" s="13" t="n"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Harbor Partners</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Comm Loan</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="n">
+        <v>15724903.49</v>
+      </c>
+      <c r="E3" s="12" t="n">
+        <v>0.0583</v>
+      </c>
+      <c r="F3" s="13" t="n">
+        <v>46126</v>
+      </c>
       <c r="G3" s="14">
         <f>IF(F3="","",TODAY()-F3)</f>
         <v/>
       </c>
-      <c r="H3" s="13" t="n"/>
+      <c r="H3" s="13" t="n">
+        <v>46378</v>
+      </c>
       <c r="I3" s="15">
         <f>IF(OR(B3="",D3=""),"",D3*VLOOKUP(B3,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -3795,20 +4539,37 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="16" t="n"/>
-      <c r="B4" s="16" t="n"/>
-      <c r="C4" s="16" t="n"/>
-      <c r="D4" s="17" t="n"/>
-      <c r="E4" s="12">
-        <f>IF(C4="","",VLOOKUP(C4,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F4" s="18" t="n"/>
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>Ironwood Capital</t>
+        </is>
+      </c>
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>Deposits</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="D4" s="17" t="n">
+        <v>933487.87</v>
+      </c>
+      <c r="E4" s="12" t="n">
+        <v>0.1089</v>
+      </c>
+      <c r="F4" s="18" t="n">
+        <v>46139</v>
+      </c>
       <c r="G4" s="14">
         <f>IF(F4="","",TODAY()-F4)</f>
         <v/>
       </c>
-      <c r="H4" s="18" t="n"/>
+      <c r="H4" s="18" t="n">
+        <v>46375</v>
+      </c>
       <c r="I4" s="15">
         <f>IF(OR(B4="",D4=""),"",D4*VLOOKUP(B4,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -3820,17 +4581,37 @@
       <c r="K4" s="16" t="n"/>
     </row>
     <row r="5">
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="12">
-        <f>IF(C5="","",VLOOKUP(C5,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F5" s="13" t="n"/>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Juniper Foods</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Comm Loan</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Proposal</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>779233.08</v>
+      </c>
+      <c r="E5" s="12" t="n">
+        <v>0.4508</v>
+      </c>
+      <c r="F5" s="13" t="n">
+        <v>46100</v>
+      </c>
       <c r="G5" s="14">
         <f>IF(F5="","",TODAY()-F5)</f>
         <v/>
       </c>
-      <c r="H5" s="13" t="n"/>
+      <c r="H5" s="13" t="n">
+        <v>46276</v>
+      </c>
       <c r="I5" s="15">
         <f>IF(OR(B5="",D5=""),"",D5*VLOOKUP(B5,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -3841,20 +4622,37 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="n"/>
-      <c r="B6" s="16" t="n"/>
-      <c r="C6" s="16" t="n"/>
-      <c r="D6" s="17" t="n"/>
-      <c r="E6" s="12">
-        <f>IF(C6="","",VLOOKUP(C6,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F6" s="18" t="n"/>
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>Keystone Steel</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>Comm Loan</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>Qualified</t>
+        </is>
+      </c>
+      <c r="D6" s="17" t="n">
+        <v>2585647.29</v>
+      </c>
+      <c r="E6" s="12" t="n">
+        <v>0.2363</v>
+      </c>
+      <c r="F6" s="18" t="n">
+        <v>46114</v>
+      </c>
       <c r="G6" s="14">
         <f>IF(F6="","",TODAY()-F6)</f>
         <v/>
       </c>
-      <c r="H6" s="18" t="n"/>
+      <c r="H6" s="18" t="n">
+        <v>46314</v>
+      </c>
       <c r="I6" s="15">
         <f>IF(OR(B6="",D6=""),"",D6*VLOOKUP(B6,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -3866,17 +4664,37 @@
       <c r="K6" s="16" t="n"/>
     </row>
     <row r="7">
-      <c r="D7" s="6" t="n"/>
-      <c r="E7" s="12">
-        <f>IF(C7="","",VLOOKUP(C7,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F7" s="13" t="n"/>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Lakeside Medical</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Comm Loan</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Qualified</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>5200728.88</v>
+      </c>
+      <c r="E7" s="12" t="n">
+        <v>0.2737</v>
+      </c>
+      <c r="F7" s="13" t="n">
+        <v>46171</v>
+      </c>
       <c r="G7" s="14">
         <f>IF(F7="","",TODAY()-F7)</f>
         <v/>
       </c>
-      <c r="H7" s="13" t="n"/>
+      <c r="H7" s="13" t="n">
+        <v>46310</v>
+      </c>
       <c r="I7" s="15">
         <f>IF(OR(B7="",D7=""),"",D7*VLOOKUP(B7,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -3887,20 +4705,37 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="n"/>
-      <c r="B8" s="16" t="n"/>
-      <c r="C8" s="16" t="n"/>
-      <c r="D8" s="17" t="n"/>
-      <c r="E8" s="12">
-        <f>IF(C8="","",VLOOKUP(C8,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F8" s="18" t="n"/>
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>Mason &amp; Co.</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>Other Fees</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="D8" s="17" t="n">
+        <v>22812.17</v>
+      </c>
+      <c r="E8" s="12" t="n">
+        <v>0.0764</v>
+      </c>
+      <c r="F8" s="18" t="n">
+        <v>46033</v>
+      </c>
       <c r="G8" s="14">
         <f>IF(F8="","",TODAY()-F8)</f>
         <v/>
       </c>
-      <c r="H8" s="18" t="n"/>
+      <c r="H8" s="18" t="n">
+        <v>46383</v>
+      </c>
       <c r="I8" s="15">
         <f>IF(OR(B8="",D8=""),"",D8*VLOOKUP(B8,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -3912,17 +4747,37 @@
       <c r="K8" s="16" t="n"/>
     </row>
     <row r="9">
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="12">
-        <f>IF(C9="","",VLOOKUP(C9,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F9" s="13" t="n"/>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Northstar Tech</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Comm Loan</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>7356362.08</v>
+      </c>
+      <c r="E9" s="12" t="n">
+        <v>0.08740000000000001</v>
+      </c>
+      <c r="F9" s="13" t="n">
+        <v>46188</v>
+      </c>
       <c r="G9" s="14">
         <f>IF(F9="","",TODAY()-F9)</f>
         <v/>
       </c>
-      <c r="H9" s="13" t="n"/>
+      <c r="H9" s="13" t="n">
+        <v>46377</v>
+      </c>
       <c r="I9" s="15">
         <f>IF(OR(B9="",D9=""),"",D9*VLOOKUP(B9,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -4584,17 +5439,37 @@
       </c>
     </row>
     <row r="3">
-      <c r="D3" s="6" t="n"/>
-      <c r="E3" s="12">
-        <f>IF(C3="","",VLOOKUP(C3,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F3" s="13" t="n"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Redwood Construction</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Comm Loan</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="n">
+        <v>17680675.93</v>
+      </c>
+      <c r="E3" s="12" t="n">
+        <v>0.7914</v>
+      </c>
+      <c r="F3" s="13" t="n">
+        <v>46142</v>
+      </c>
       <c r="G3" s="14">
         <f>IF(F3="","",TODAY()-F3)</f>
         <v/>
       </c>
-      <c r="H3" s="13" t="n"/>
+      <c r="H3" s="13" t="n">
+        <v>46261</v>
+      </c>
       <c r="I3" s="15">
         <f>IF(OR(B3="",D3=""),"",D3*VLOOKUP(B3,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -4605,20 +5480,37 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="16" t="n"/>
-      <c r="B4" s="16" t="n"/>
-      <c r="C4" s="16" t="n"/>
-      <c r="D4" s="17" t="n"/>
-      <c r="E4" s="12">
-        <f>IF(C4="","",VLOOKUP(C4,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F4" s="18" t="n"/>
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>Summit Hospitality</t>
+        </is>
+      </c>
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>Comm Loan</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="inlineStr">
+        <is>
+          <t>Proposal</t>
+        </is>
+      </c>
+      <c r="D4" s="17" t="n">
+        <v>2595942.77</v>
+      </c>
+      <c r="E4" s="12" t="n">
+        <v>0.4503</v>
+      </c>
+      <c r="F4" s="18" t="n">
+        <v>46142</v>
+      </c>
       <c r="G4" s="14">
         <f>IF(F4="","",TODAY()-F4)</f>
         <v/>
       </c>
-      <c r="H4" s="18" t="n"/>
+      <c r="H4" s="18" t="n">
+        <v>46307</v>
+      </c>
       <c r="I4" s="15">
         <f>IF(OR(B4="",D4=""),"",D4*VLOOKUP(B4,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -4630,17 +5522,37 @@
       <c r="K4" s="16" t="n"/>
     </row>
     <row r="5">
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="12">
-        <f>IF(C5="","",VLOOKUP(C5,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F5" s="13" t="n"/>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Trinity Pharma</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Comm Loan</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>10550099.4</v>
+      </c>
+      <c r="E5" s="12" t="n">
+        <v>0.0508</v>
+      </c>
+      <c r="F5" s="13" t="n">
+        <v>46137</v>
+      </c>
       <c r="G5" s="14">
         <f>IF(F5="","",TODAY()-F5)</f>
         <v/>
       </c>
-      <c r="H5" s="13" t="n"/>
+      <c r="H5" s="13" t="n">
+        <v>46352</v>
+      </c>
       <c r="I5" s="15">
         <f>IF(OR(B5="",D5=""),"",D5*VLOOKUP(B5,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -4651,20 +5563,37 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="n"/>
-      <c r="B6" s="16" t="n"/>
-      <c r="C6" s="16" t="n"/>
-      <c r="D6" s="17" t="n"/>
-      <c r="E6" s="12">
-        <f>IF(C6="","",VLOOKUP(C6,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F6" s="18" t="n"/>
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>Union Distributors</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>Deposits</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>Qualified</t>
+        </is>
+      </c>
+      <c r="D6" s="17" t="n">
+        <v>1055220.28</v>
+      </c>
+      <c r="E6" s="12" t="n">
+        <v>0.2275</v>
+      </c>
+      <c r="F6" s="18" t="n">
+        <v>46182</v>
+      </c>
       <c r="G6" s="14">
         <f>IF(F6="","",TODAY()-F6)</f>
         <v/>
       </c>
-      <c r="H6" s="18" t="n"/>
+      <c r="H6" s="18" t="n">
+        <v>46337</v>
+      </c>
       <c r="I6" s="15">
         <f>IF(OR(B6="",D6=""),"",D6*VLOOKUP(B6,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -4676,17 +5605,37 @@
       <c r="K6" s="16" t="n"/>
     </row>
     <row r="7">
-      <c r="D7" s="6" t="n"/>
-      <c r="E7" s="12">
-        <f>IF(C7="","",VLOOKUP(C7,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F7" s="13" t="n"/>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Vanguard Plastics</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Deposits</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Qualified</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>4639920.43</v>
+      </c>
+      <c r="E7" s="12" t="n">
+        <v>0.2146</v>
+      </c>
+      <c r="F7" s="13" t="n">
+        <v>46126</v>
+      </c>
       <c r="G7" s="14">
         <f>IF(F7="","",TODAY()-F7)</f>
         <v/>
       </c>
-      <c r="H7" s="13" t="n"/>
+      <c r="H7" s="13" t="n">
+        <v>46330</v>
+      </c>
       <c r="I7" s="15">
         <f>IF(OR(B7="",D7=""),"",D7*VLOOKUP(B7,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -4697,20 +5646,37 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="n"/>
-      <c r="B8" s="16" t="n"/>
-      <c r="C8" s="16" t="n"/>
-      <c r="D8" s="17" t="n"/>
-      <c r="E8" s="12">
-        <f>IF(C8="","",VLOOKUP(C8,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F8" s="18" t="n"/>
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>Westfield Retail</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>Comm Loan</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="D8" s="17" t="n">
+        <v>1585817.67</v>
+      </c>
+      <c r="E8" s="12" t="n">
+        <v>0.1178</v>
+      </c>
+      <c r="F8" s="18" t="n">
+        <v>46167</v>
+      </c>
       <c r="G8" s="14">
         <f>IF(F8="","",TODAY()-F8)</f>
         <v/>
       </c>
-      <c r="H8" s="18" t="n"/>
+      <c r="H8" s="18" t="n">
+        <v>46331</v>
+      </c>
       <c r="I8" s="15">
         <f>IF(OR(B8="",D8=""),"",D8*VLOOKUP(B8,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -4722,17 +5688,37 @@
       <c r="K8" s="16" t="n"/>
     </row>
     <row r="9">
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="12">
-        <f>IF(C9="","",VLOOKUP(C9,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F9" s="13" t="n"/>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Xander Aviation</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Comm Loan</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>2728841.32</v>
+      </c>
+      <c r="E9" s="12" t="n">
+        <v>0.1017</v>
+      </c>
+      <c r="F9" s="13" t="n">
+        <v>46182</v>
+      </c>
       <c r="G9" s="14">
         <f>IF(F9="","",TODAY()-F9)</f>
         <v/>
       </c>
-      <c r="H9" s="13" t="n"/>
+      <c r="H9" s="13" t="n">
+        <v>46363</v>
+      </c>
       <c r="I9" s="15">
         <f>IF(OR(B9="",D9=""),"",D9*VLOOKUP(B9,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -4743,20 +5729,37 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="n"/>
-      <c r="B10" s="16" t="n"/>
-      <c r="C10" s="16" t="n"/>
-      <c r="D10" s="17" t="n"/>
-      <c r="E10" s="12">
-        <f>IF(C10="","",VLOOKUP(C10,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F10" s="18" t="n"/>
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t>Yellowstone Ranch</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>Other Fees</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="inlineStr">
+        <is>
+          <t>Proposal</t>
+        </is>
+      </c>
+      <c r="D10" s="17" t="n">
+        <v>24484.22</v>
+      </c>
+      <c r="E10" s="12" t="n">
+        <v>0.4725</v>
+      </c>
+      <c r="F10" s="18" t="n">
+        <v>46115</v>
+      </c>
       <c r="G10" s="14">
         <f>IF(F10="","",TODAY()-F10)</f>
         <v/>
       </c>
-      <c r="H10" s="18" t="n"/>
+      <c r="H10" s="18" t="n">
+        <v>46270</v>
+      </c>
       <c r="I10" s="15">
         <f>IF(OR(B10="",D10=""),"",D10*VLOOKUP(B10,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -4768,17 +5771,37 @@
       <c r="K10" s="16" t="n"/>
     </row>
     <row r="11">
-      <c r="D11" s="6" t="n"/>
-      <c r="E11" s="12">
-        <f>IF(C11="","",VLOOKUP(C11,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F11" s="13" t="n"/>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Zenith Software</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Deposits</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>3267346.24</v>
+      </c>
+      <c r="E11" s="12" t="n">
+        <v>0.117</v>
+      </c>
+      <c r="F11" s="13" t="n">
+        <v>46162</v>
+      </c>
       <c r="G11" s="14">
         <f>IF(F11="","",TODAY()-F11)</f>
         <v/>
       </c>
-      <c r="H11" s="13" t="n"/>
+      <c r="H11" s="13" t="n">
+        <v>46333</v>
+      </c>
       <c r="I11" s="15">
         <f>IF(OR(B11="",D11=""),"",D11*VLOOKUP(B11,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -5394,17 +6417,37 @@
       </c>
     </row>
     <row r="3">
-      <c r="D3" s="6" t="n"/>
-      <c r="E3" s="12">
-        <f>IF(C3="","",VLOOKUP(C3,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F3" s="13" t="n"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Union Distributors</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Other Fees</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Qualified</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="n">
+        <v>49498.92</v>
+      </c>
+      <c r="E3" s="12" t="n">
+        <v>0.2127</v>
+      </c>
+      <c r="F3" s="13" t="n">
+        <v>46081</v>
+      </c>
       <c r="G3" s="14">
         <f>IF(F3="","",TODAY()-F3)</f>
         <v/>
       </c>
-      <c r="H3" s="13" t="n"/>
+      <c r="H3" s="13" t="n">
+        <v>46337</v>
+      </c>
       <c r="I3" s="15">
         <f>IF(OR(B3="",D3=""),"",D3*VLOOKUP(B3,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -5415,20 +6458,37 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="16" t="n"/>
-      <c r="B4" s="16" t="n"/>
-      <c r="C4" s="16" t="n"/>
-      <c r="D4" s="17" t="n"/>
-      <c r="E4" s="12">
-        <f>IF(C4="","",VLOOKUP(C4,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F4" s="18" t="n"/>
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>Vanguard Plastics</t>
+        </is>
+      </c>
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>Treasury Mgmt</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="D4" s="17" t="n">
+        <v>117786.33</v>
+      </c>
+      <c r="E4" s="12" t="n">
+        <v>0.1338</v>
+      </c>
+      <c r="F4" s="18" t="n">
+        <v>46143</v>
+      </c>
       <c r="G4" s="14">
         <f>IF(F4="","",TODAY()-F4)</f>
         <v/>
       </c>
-      <c r="H4" s="18" t="n"/>
+      <c r="H4" s="18" t="n">
+        <v>46376</v>
+      </c>
       <c r="I4" s="15">
         <f>IF(OR(B4="",D4=""),"",D4*VLOOKUP(B4,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -5440,17 +6500,37 @@
       <c r="K4" s="16" t="n"/>
     </row>
     <row r="5">
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="12">
-        <f>IF(C5="","",VLOOKUP(C5,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F5" s="13" t="n"/>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Westfield Retail</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Comm Loan</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>3693911.73</v>
+      </c>
+      <c r="E5" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="13" t="n">
+        <v>46098</v>
+      </c>
       <c r="G5" s="14">
         <f>IF(F5="","",TODAY()-F5)</f>
         <v/>
       </c>
-      <c r="H5" s="13" t="n"/>
+      <c r="H5" s="13" t="n">
+        <v>46213</v>
+      </c>
       <c r="I5" s="15">
         <f>IF(OR(B5="",D5=""),"",D5*VLOOKUP(B5,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -5461,20 +6541,37 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="n"/>
-      <c r="B6" s="16" t="n"/>
-      <c r="C6" s="16" t="n"/>
-      <c r="D6" s="17" t="n"/>
-      <c r="E6" s="12">
-        <f>IF(C6="","",VLOOKUP(C6,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F6" s="18" t="n"/>
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>Xander Aviation</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>Other Fees</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="D6" s="17" t="n">
+        <v>40457.68</v>
+      </c>
+      <c r="E6" s="12" t="n">
+        <v>0.1036</v>
+      </c>
+      <c r="F6" s="18" t="n">
+        <v>46135</v>
+      </c>
       <c r="G6" s="14">
         <f>IF(F6="","",TODAY()-F6)</f>
         <v/>
       </c>
-      <c r="H6" s="18" t="n"/>
+      <c r="H6" s="18" t="n">
+        <v>46383</v>
+      </c>
       <c r="I6" s="15">
         <f>IF(OR(B6="",D6=""),"",D6*VLOOKUP(B6,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -5486,17 +6583,37 @@
       <c r="K6" s="16" t="n"/>
     </row>
     <row r="7">
-      <c r="D7" s="6" t="n"/>
-      <c r="E7" s="12">
-        <f>IF(C7="","",VLOOKUP(C7,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F7" s="13" t="n"/>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Yellowstone Ranch</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Comm Loan</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Qualified</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>2322589.74</v>
+      </c>
+      <c r="E7" s="12" t="n">
+        <v>0.2114</v>
+      </c>
+      <c r="F7" s="13" t="n">
+        <v>46078</v>
+      </c>
       <c r="G7" s="14">
         <f>IF(F7="","",TODAY()-F7)</f>
         <v/>
       </c>
-      <c r="H7" s="13" t="n"/>
+      <c r="H7" s="13" t="n">
+        <v>46343</v>
+      </c>
       <c r="I7" s="15">
         <f>IF(OR(B7="",D7=""),"",D7*VLOOKUP(B7,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -5507,20 +6624,37 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="n"/>
-      <c r="B8" s="16" t="n"/>
-      <c r="C8" s="16" t="n"/>
-      <c r="D8" s="17" t="n"/>
-      <c r="E8" s="12">
-        <f>IF(C8="","",VLOOKUP(C8,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F8" s="18" t="n"/>
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>Zenith Software</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>Deposits</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>Proposal</t>
+        </is>
+      </c>
+      <c r="D8" s="17" t="n">
+        <v>5664478.31</v>
+      </c>
+      <c r="E8" s="12" t="n">
+        <v>0.5112</v>
+      </c>
+      <c r="F8" s="18" t="n">
+        <v>46151</v>
+      </c>
       <c r="G8" s="14">
         <f>IF(F8="","",TODAY()-F8)</f>
         <v/>
       </c>
-      <c r="H8" s="18" t="n"/>
+      <c r="H8" s="18" t="n">
+        <v>46299</v>
+      </c>
       <c r="I8" s="15">
         <f>IF(OR(B8="",D8=""),"",D8*VLOOKUP(B8,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -5532,17 +6666,37 @@
       <c r="K8" s="16" t="n"/>
     </row>
     <row r="9">
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="12">
-        <f>IF(C9="","",VLOOKUP(C9,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F9" s="13" t="n"/>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Alamo Equipment</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Treasury Mgmt</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>250208.93</v>
+      </c>
+      <c r="E9" s="12" t="n">
+        <v>0.8488</v>
+      </c>
+      <c r="F9" s="13" t="n">
+        <v>46131</v>
+      </c>
       <c r="G9" s="14">
         <f>IF(F9="","",TODAY()-F9)</f>
         <v/>
       </c>
-      <c r="H9" s="13" t="n"/>
+      <c r="H9" s="13" t="n">
+        <v>46269</v>
+      </c>
       <c r="I9" s="15">
         <f>IF(OR(B9="",D9=""),"",D9*VLOOKUP(B9,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -6204,17 +7358,37 @@
       </c>
     </row>
     <row r="3">
-      <c r="D3" s="6" t="n"/>
-      <c r="E3" s="12">
-        <f>IF(C3="","",VLOOKUP(C3,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F3" s="13" t="n"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Evergreen Realty</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Deposits</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Qualified</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="n">
+        <v>4276478.29</v>
+      </c>
+      <c r="E3" s="12" t="n">
+        <v>0.2008</v>
+      </c>
+      <c r="F3" s="13" t="n">
+        <v>46129</v>
+      </c>
       <c r="G3" s="14">
         <f>IF(F3="","",TODAY()-F3)</f>
         <v/>
       </c>
-      <c r="H3" s="13" t="n"/>
+      <c r="H3" s="13" t="n">
+        <v>46339</v>
+      </c>
       <c r="I3" s="15">
         <f>IF(OR(B3="",D3=""),"",D3*VLOOKUP(B3,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -6225,20 +7399,37 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="16" t="n"/>
-      <c r="B4" s="16" t="n"/>
-      <c r="C4" s="16" t="n"/>
-      <c r="D4" s="17" t="n"/>
-      <c r="E4" s="12">
-        <f>IF(C4="","",VLOOKUP(C4,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F4" s="18" t="n"/>
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>Fairfield Energy</t>
+        </is>
+      </c>
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>Other Fees</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="D4" s="17" t="n">
+        <v>71443.88</v>
+      </c>
+      <c r="E4" s="12" t="n">
+        <v>0.8062</v>
+      </c>
+      <c r="F4" s="18" t="n">
+        <v>46156</v>
+      </c>
       <c r="G4" s="14">
         <f>IF(F4="","",TODAY()-F4)</f>
         <v/>
       </c>
-      <c r="H4" s="18" t="n"/>
+      <c r="H4" s="18" t="n">
+        <v>46285</v>
+      </c>
       <c r="I4" s="15">
         <f>IF(OR(B4="",D4=""),"",D4*VLOOKUP(B4,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -6250,17 +7441,37 @@
       <c r="K4" s="16" t="n"/>
     </row>
     <row r="5">
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="12">
-        <f>IF(C5="","",VLOOKUP(C5,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F5" s="13" t="n"/>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Galleon Logistics</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Comm Loan</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Proposal</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>3318345.97</v>
+      </c>
+      <c r="E5" s="12" t="n">
+        <v>0.5425</v>
+      </c>
+      <c r="F5" s="13" t="n">
+        <v>46158</v>
+      </c>
       <c r="G5" s="14">
         <f>IF(F5="","",TODAY()-F5)</f>
         <v/>
       </c>
-      <c r="H5" s="13" t="n"/>
+      <c r="H5" s="13" t="n">
+        <v>46302</v>
+      </c>
       <c r="I5" s="15">
         <f>IF(OR(B5="",D5=""),"",D5*VLOOKUP(B5,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -6271,20 +7482,37 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="n"/>
-      <c r="B6" s="16" t="n"/>
-      <c r="C6" s="16" t="n"/>
-      <c r="D6" s="17" t="n"/>
-      <c r="E6" s="12">
-        <f>IF(C6="","",VLOOKUP(C6,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F6" s="18" t="n"/>
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>Harbor Partners</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>Deposits</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="D6" s="17" t="n">
+        <v>942755.35</v>
+      </c>
+      <c r="E6" s="12" t="n">
+        <v>0.0574</v>
+      </c>
+      <c r="F6" s="18" t="n">
+        <v>46118</v>
+      </c>
       <c r="G6" s="14">
         <f>IF(F6="","",TODAY()-F6)</f>
         <v/>
       </c>
-      <c r="H6" s="18" t="n"/>
+      <c r="H6" s="18" t="n">
+        <v>46337</v>
+      </c>
       <c r="I6" s="15">
         <f>IF(OR(B6="",D6=""),"",D6*VLOOKUP(B6,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -6296,17 +7524,37 @@
       <c r="K6" s="16" t="n"/>
     </row>
     <row r="7">
-      <c r="D7" s="6" t="n"/>
-      <c r="E7" s="12">
-        <f>IF(C7="","",VLOOKUP(C7,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F7" s="13" t="n"/>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Ironwood Capital</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Deposits</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Qualified</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>907319.76</v>
+      </c>
+      <c r="E7" s="12" t="n">
+        <v>0.2669</v>
+      </c>
+      <c r="F7" s="13" t="n">
+        <v>46169</v>
+      </c>
       <c r="G7" s="14">
         <f>IF(F7="","",TODAY()-F7)</f>
         <v/>
       </c>
-      <c r="H7" s="13" t="n"/>
+      <c r="H7" s="13" t="n">
+        <v>46314</v>
+      </c>
       <c r="I7" s="15">
         <f>IF(OR(B7="",D7=""),"",D7*VLOOKUP(B7,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -6317,20 +7565,37 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="n"/>
-      <c r="B8" s="16" t="n"/>
-      <c r="C8" s="16" t="n"/>
-      <c r="D8" s="17" t="n"/>
-      <c r="E8" s="12">
-        <f>IF(C8="","",VLOOKUP(C8,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F8" s="18" t="n"/>
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>Juniper Foods</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>Comm Loan</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>Qualified</t>
+        </is>
+      </c>
+      <c r="D8" s="17" t="n">
+        <v>14970368.89</v>
+      </c>
+      <c r="E8" s="12" t="n">
+        <v>0.2907</v>
+      </c>
+      <c r="F8" s="18" t="n">
+        <v>46168</v>
+      </c>
       <c r="G8" s="14">
         <f>IF(F8="","",TODAY()-F8)</f>
         <v/>
       </c>
-      <c r="H8" s="18" t="n"/>
+      <c r="H8" s="18" t="n">
+        <v>46312</v>
+      </c>
       <c r="I8" s="15">
         <f>IF(OR(B8="",D8=""),"",D8*VLOOKUP(B8,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -6342,17 +7607,37 @@
       <c r="K8" s="16" t="n"/>
     </row>
     <row r="9">
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="12">
-        <f>IF(C9="","",VLOOKUP(C9,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F9" s="13" t="n"/>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Keystone Steel</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Deposits</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Proposal</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>7146028.97</v>
+      </c>
+      <c r="E9" s="12" t="n">
+        <v>0.4834</v>
+      </c>
+      <c r="F9" s="13" t="n">
+        <v>46135</v>
+      </c>
       <c r="G9" s="14">
         <f>IF(F9="","",TODAY()-F9)</f>
         <v/>
       </c>
-      <c r="H9" s="13" t="n"/>
+      <c r="H9" s="13" t="n">
+        <v>46304</v>
+      </c>
       <c r="I9" s="15">
         <f>IF(OR(B9="",D9=""),"",D9*VLOOKUP(B9,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -6363,20 +7648,37 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="n"/>
-      <c r="B10" s="16" t="n"/>
-      <c r="C10" s="16" t="n"/>
-      <c r="D10" s="17" t="n"/>
-      <c r="E10" s="12">
-        <f>IF(C10="","",VLOOKUP(C10,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F10" s="18" t="n"/>
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t>Lakeside Medical</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>Treasury Mgmt</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="D10" s="17" t="n">
+        <v>36610.28</v>
+      </c>
+      <c r="E10" s="12" t="n">
+        <v>0.9827</v>
+      </c>
+      <c r="F10" s="18" t="n">
+        <v>46189</v>
+      </c>
       <c r="G10" s="14">
         <f>IF(F10="","",TODAY()-F10)</f>
         <v/>
       </c>
-      <c r="H10" s="18" t="n"/>
+      <c r="H10" s="18" t="n">
+        <v>46240</v>
+      </c>
       <c r="I10" s="15">
         <f>IF(OR(B10="",D10=""),"",D10*VLOOKUP(B10,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -6388,17 +7690,37 @@
       <c r="K10" s="16" t="n"/>
     </row>
     <row r="11">
-      <c r="D11" s="6" t="n"/>
-      <c r="E11" s="12">
-        <f>IF(C11="","",VLOOKUP(C11,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F11" s="13" t="n"/>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Mason &amp; Co.</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Comm Loan</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Proposal</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>3839311.46</v>
+      </c>
+      <c r="E11" s="12" t="n">
+        <v>0.4668</v>
+      </c>
+      <c r="F11" s="13" t="n">
+        <v>46181</v>
+      </c>
       <c r="G11" s="14">
         <f>IF(F11="","",TODAY()-F11)</f>
         <v/>
       </c>
-      <c r="H11" s="13" t="n"/>
+      <c r="H11" s="13" t="n">
+        <v>46279</v>
+      </c>
       <c r="I11" s="15">
         <f>IF(OR(B11="",D11=""),"",D11*VLOOKUP(B11,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -6409,20 +7731,37 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="16" t="n"/>
-      <c r="B12" s="16" t="n"/>
-      <c r="C12" s="16" t="n"/>
-      <c r="D12" s="17" t="n"/>
-      <c r="E12" s="12">
-        <f>IF(C12="","",VLOOKUP(C12,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F12" s="18" t="n"/>
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>Northstar Tech</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>Comm Loan</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>Proposal</t>
+        </is>
+      </c>
+      <c r="D12" s="17" t="n">
+        <v>18165595.86</v>
+      </c>
+      <c r="E12" s="12" t="n">
+        <v>0.5009</v>
+      </c>
+      <c r="F12" s="18" t="n">
+        <v>46163</v>
+      </c>
       <c r="G12" s="14">
         <f>IF(F12="","",TODAY()-F12)</f>
         <v/>
       </c>
-      <c r="H12" s="18" t="n"/>
+      <c r="H12" s="18" t="n">
+        <v>46301</v>
+      </c>
       <c r="I12" s="15">
         <f>IF(OR(B12="",D12=""),"",D12*VLOOKUP(B12,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -6434,17 +7773,37 @@
       <c r="K12" s="16" t="n"/>
     </row>
     <row r="13">
-      <c r="D13" s="6" t="n"/>
-      <c r="E13" s="12">
-        <f>IF(C13="","",VLOOKUP(C13,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F13" s="13" t="n"/>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Xander Aviation</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Treasury Mgmt</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>101352.17</v>
+      </c>
+      <c r="E13" s="12" t="n">
+        <v>0.0709</v>
+      </c>
+      <c r="F13" s="13" t="n">
+        <v>46153</v>
+      </c>
       <c r="G13" s="14">
         <f>IF(F13="","",TODAY()-F13)</f>
         <v/>
       </c>
-      <c r="H13" s="13" t="n"/>
+      <c r="H13" s="13" t="n">
+        <v>46354</v>
+      </c>
       <c r="I13" s="15">
         <f>IF(OR(B13="",D13=""),"",D13*VLOOKUP(B13,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -6455,20 +7814,37 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="16" t="n"/>
-      <c r="B14" s="16" t="n"/>
-      <c r="C14" s="16" t="n"/>
-      <c r="D14" s="17" t="n"/>
-      <c r="E14" s="12">
-        <f>IF(C14="","",VLOOKUP(C14,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F14" s="18" t="n"/>
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>Yellowstone Ranch</t>
+        </is>
+      </c>
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>Other Fees</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="D14" s="17" t="n">
+        <v>4379.97</v>
+      </c>
+      <c r="E14" s="12" t="n">
+        <v>0.08019999999999999</v>
+      </c>
+      <c r="F14" s="18" t="n">
+        <v>46120</v>
+      </c>
       <c r="G14" s="14">
         <f>IF(F14="","",TODAY()-F14)</f>
         <v/>
       </c>
-      <c r="H14" s="18" t="n"/>
+      <c r="H14" s="18" t="n">
+        <v>46354</v>
+      </c>
       <c r="I14" s="15">
         <f>IF(OR(B14="",D14=""),"",D14*VLOOKUP(B14,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -6480,17 +7856,37 @@
       <c r="K14" s="16" t="n"/>
     </row>
     <row r="15">
-      <c r="D15" s="6" t="n"/>
-      <c r="E15" s="12">
-        <f>IF(C15="","",VLOOKUP(C15,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F15" s="13" t="n"/>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Zenith Software</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Comm Loan</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>9360282.949999999</v>
+      </c>
+      <c r="E15" s="12" t="n">
+        <v>0.751</v>
+      </c>
+      <c r="F15" s="13" t="n">
+        <v>46160</v>
+      </c>
       <c r="G15" s="14">
         <f>IF(F15="","",TODAY()-F15)</f>
         <v/>
       </c>
-      <c r="H15" s="13" t="n"/>
+      <c r="H15" s="13" t="n">
+        <v>46247</v>
+      </c>
       <c r="I15" s="15">
         <f>IF(OR(B15="",D15=""),"",D15*VLOOKUP(B15,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>
@@ -6501,20 +7897,37 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="16" t="n"/>
-      <c r="B16" s="16" t="n"/>
-      <c r="C16" s="16" t="n"/>
-      <c r="D16" s="17" t="n"/>
-      <c r="E16" s="12">
-        <f>IF(C16="","",VLOOKUP(C16,Lookup!$D$2:$E$6,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F16" s="18" t="n"/>
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>Alamo Equipment</t>
+        </is>
+      </c>
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>Deposits</t>
+        </is>
+      </c>
+      <c r="C16" s="16" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="D16" s="17" t="n">
+        <v>1565237.54</v>
+      </c>
+      <c r="E16" s="12" t="n">
+        <v>0.9879</v>
+      </c>
+      <c r="F16" s="18" t="n">
+        <v>46148</v>
+      </c>
       <c r="G16" s="14">
         <f>IF(F16="","",TODAY()-F16)</f>
         <v/>
       </c>
-      <c r="H16" s="18" t="n"/>
+      <c r="H16" s="18" t="n">
+        <v>46224</v>
+      </c>
       <c r="I16" s="15">
         <f>IF(OR(B16="",D16=""),"",D16*VLOOKUP(B16,Lookup!$A$2:$B$5,2,FALSE))</f>
         <v/>

</xml_diff>